<commit_message>
feat: rectified open api spec and renamed API
</commit_message>
<xml_diff>
--- a/data/gst/schema/public/unregistered-applicants-validation/v1.0/fields.xlsx
+++ b/data/gst/schema/public/unregistered-applicants-validation/v1.0/fields.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="36">
   <si>
     <t>Parameter Name</t>
   </si>
@@ -132,6 +132,12 @@
   </si>
   <si>
     <t>TP</t>
+  </si>
+  <si>
+    <t>uid</t>
+  </si>
+  <si>
+    <t>UID of the Unregistered Applicants</t>
   </si>
 </sst>
 </file>
@@ -726,9 +732,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns4="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.5" ns3:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21.81640625" customWidth="1"/>
     <col min="2" max="2" width="43.7265625" customWidth="1"/>
@@ -738,7 +744,7 @@
     <col min="6" max="6" width="23.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" ns3:dyDescent="0.35">
       <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
@@ -758,7 +764,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:6" s="30" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" s="30" customFormat="1" ns3:dyDescent="0.35">
       <c r="A2" s="31" t="s">
         <v>31</v>
       </c>
@@ -778,12 +784,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" ns3:dyDescent="0.35">
       <c r="A3" s="19" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="B3" s="29" t="s">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="C3" s="29" t="s">
         <v>5</v>
@@ -798,7 +804,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" ht="29" ns3:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>26</v>
       </c>
@@ -818,7 +824,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" ht="29" ns3:dyDescent="0.35">
       <c r="A5" s="43" t="s">
         <v>27</v>
       </c>
@@ -838,7 +844,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" ns3:dyDescent="0.35">
       <c r="A6" s="1"/>
       <c r="B6" s="4"/>
       <c r="C6" s="2"/>
@@ -846,7 +852,7 @@
       <c r="E6" s="3"/>
       <c r="F6" s="8"/>
     </row>
-    <row r="7" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" ht="21" customHeight="1" ns3:dyDescent="0.35">
       <c r="A7" s="24" t="s">
         <v>30</v>
       </c>
@@ -856,7 +862,7 @@
       <c r="E7" s="25"/>
       <c r="F7" s="25"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" ns3:dyDescent="0.35">
       <c r="A8" s="1"/>
       <c r="B8" s="4"/>
       <c r="C8" s="2"/>
@@ -864,91 +870,91 @@
       <c r="E8" s="9"/>
       <c r="F8" s="8"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" ns3:dyDescent="0.35">
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
       <c r="C9" s="5"/>
       <c r="D9" s="6"/>
       <c r="E9" s="6"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" ns3:dyDescent="0.35">
       <c r="A10" s="6"/>
       <c r="B10" s="6"/>
       <c r="C10" s="7"/>
       <c r="D10" s="6"/>
       <c r="E10" s="6"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" ns3:dyDescent="0.35">
       <c r="A11" s="6"/>
       <c r="B11" s="6"/>
       <c r="C11" s="18"/>
       <c r="D11" s="6"/>
       <c r="E11" s="6"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" ns3:dyDescent="0.35">
       <c r="A12" s="6"/>
       <c r="B12" s="6"/>
       <c r="C12" s="7"/>
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" ns3:dyDescent="0.35">
       <c r="A13" s="6"/>
       <c r="B13" s="6"/>
       <c r="C13" s="7"/>
       <c r="D13" s="6"/>
       <c r="E13" s="6"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" ns3:dyDescent="0.35">
       <c r="A14" s="6"/>
       <c r="B14" s="6"/>
       <c r="C14" s="7"/>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" ns3:dyDescent="0.35">
       <c r="A15" s="6"/>
       <c r="B15" s="6"/>
       <c r="C15" s="7"/>
       <c r="D15" s="6"/>
       <c r="E15" s="6"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" ns3:dyDescent="0.35">
       <c r="A16" s="6"/>
       <c r="B16" s="6"/>
       <c r="C16" s="7"/>
       <c r="D16" s="6"/>
       <c r="E16" s="6"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" ns3:dyDescent="0.35">
       <c r="A17" s="6"/>
       <c r="B17" s="6"/>
       <c r="C17" s="7"/>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" ns3:dyDescent="0.35">
       <c r="A18" s="6"/>
       <c r="B18" s="6"/>
       <c r="C18" s="7"/>
       <c r="D18" s="6"/>
       <c r="E18" s="6"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" ns3:dyDescent="0.35">
       <c r="A19" s="6"/>
       <c r="B19" s="6"/>
       <c r="C19" s="7"/>
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" ns3:dyDescent="0.35">
       <c r="A20" s="6"/>
       <c r="B20" s="6"/>
       <c r="C20" s="7"/>
       <c r="D20" s="6"/>
       <c r="E20" s="6"/>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" ns3:dyDescent="0.35">
       <c r="A21" s="10"/>
       <c r="B21" s="10"/>
       <c r="C21" s="11"/>
@@ -959,10 +965,10 @@
     <mergeCell ref="A7:F7"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="E5" r:id="rId1" xr:uid="{AD97D8D6-FC67-41B4-A135-4BC44C8E271D}"/>
+    <hyperlink ref="E5" ns4:id="rId1" ns2:uid="{AD97D8D6-FC67-41B4-A135-4BC44C8E271D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
+  <pageSetup orientation="portrait" ns4:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
chore: updated from uid to enrolment number
</commit_message>
<xml_diff>
--- a/data/gst/schema/public/unregistered-applicants-validation/v1.0/fields.xlsx
+++ b/data/gst/schema/public/unregistered-applicants-validation/v1.0/fields.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="37">
   <si>
     <t>Parameter Name</t>
   </si>
@@ -138,6 +138,9 @@
   </si>
   <si>
     <t>UID of the Unregistered Applicants</t>
+  </si>
+  <si>
+    <t>Enrolment Number of the Unregistered Applicant</t>
   </si>
 </sst>
 </file>
@@ -786,10 +789,10 @@
     </row>
     <row r="3" spans="1:6" ns3:dyDescent="0.35">
       <c r="A3" s="19" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="B3" s="29" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C3" s="29" t="s">
         <v>5</v>

</xml_diff>